<commit_message>
Rename to Exotic Ranch & Wildlife Network; wildlife silhouette banner; giraffe favicon; remove horn logo
</commit_message>
<xml_diff>
--- a/site/downloads/herd-cashflow-roi.xlsx
+++ b/site/downloads/herd-cashflow-roi.xlsx
@@ -561,7 +561,7 @@
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>Lone Star Exotics Hub price tracker (cited sources per data point): ../prices.html and data/prices.csv</t>
+          <t>Exotic Ranch &amp; Wildlife Network price tracker (cited sources per data point): ../prices.html and data/prices.csv</t>
         </is>
       </c>
     </row>
@@ -585,7 +585,7 @@
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>Built by Lone Star Exotics Hub (draft), Oct 2026. Verify every figure against the current publication; tax law changes.</t>
+          <t>Built by Exotic Ranch &amp; Wildlife Network (draft), Oct 2026. Verify every figure against the current publication; tax law changes.</t>
         </is>
       </c>
     </row>
@@ -1760,7 +1760,6 @@
           <t>NOT tax, legal or investment advice. Educational template only. Consult a CPA and your county appraisal district.</t>
         </is>
       </c>
-      <c r="B1" s="9" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="10" t="inlineStr">

</xml_diff>